<commit_message>
docs(excel):actualizacion excel de encuestas
</commit_message>
<xml_diff>
--- a/docs/Encuesta economía (Respuestas).xlsx
+++ b/docs/Encuesta economía (Respuestas).xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="52">
   <si>
     <t>Marca temporal</t>
   </si>
@@ -152,6 +152,21 @@
   </si>
   <si>
     <t xml:space="preserve">Nunca </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Naira Villagra </t>
+  </si>
+  <si>
+    <t>Si, re</t>
+  </si>
+  <si>
+    <t>Tamara Piccinni</t>
+  </si>
+  <si>
+    <t>Este mes</t>
+  </si>
+  <si>
+    <t>si</t>
   </si>
 </sst>
 </file>
@@ -292,7 +307,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H21" displayName="Form_Responses" name="Form_Responses" id="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:H23" displayName="Form_Responses" name="Form_Responses" id="1">
   <tableColumns count="8">
     <tableColumn name="Marca temporal" id="1"/>
     <tableColumn name="Ingrese su nombre y apellido" id="2"/>
@@ -1024,6 +1039,58 @@
         <v>1.0</v>
       </c>
     </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="6">
+        <v>46162.84498616898</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C22" s="7">
+        <v>18.0</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="F22" s="7">
+        <v>4.0</v>
+      </c>
+      <c r="G22" s="7">
+        <v>5.0</v>
+      </c>
+      <c r="H22" s="7">
+        <v>2.0</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="6">
+        <v>46163.35882376158</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="C23" s="7">
+        <v>41.0</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" s="7">
+        <v>3.0</v>
+      </c>
+      <c r="G23" s="7">
+        <v>2.0</v>
+      </c>
+      <c r="H23" s="7">
+        <v>3.0</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
   <tableParts count="1">

</xml_diff>